<commit_message>
more solid project management tracking
</commit_message>
<xml_diff>
--- a/docs/stakeholder-report.xlsx
+++ b/docs/stakeholder-report.xlsx
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-03 08:12 UTC  |  matdevstamp/inl-3-awesome-journal</t>
+          <t>Generated 2026-09-03 08:13 UTC  |  matdevstamp/inl-3-awesome-journal</t>
         </is>
       </c>
     </row>
@@ -998,36 +998,36 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>What changed</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Before</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>After</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>No changes since the previous export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>What changed</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Before</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>After</t>
         </is>
       </c>
     </row>

</xml_diff>